<commit_message>
Bauhaus-Liste: dritte Hutschiene (größeres Gehäuse)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BNvKHpLgoxQiSKskTUqmN
</commit_message>
<xml_diff>
--- a/listen/Bauhaus_Einkaufsliste_MF70.xlsx
+++ b/listen/Bauhaus_Einkaufsliste_MF70.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preise: Online-Preise von bauhaus.info (Stand Dokument 04: 22.10.2026, Liste erzeugt am 22.10.2026). Im Markt können Preis und Bestand abweichen.</t>
+          <t>Preise: Online-Preise von bauhaus.info (Stand Dokument 04: 22.10.2026, Liste erzeugt am 23.10.2026). Im Markt können Preis und Bestand abweichen.</t>
         </is>
       </c>
     </row>
@@ -847,11 +847,11 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>2 Stück</t>
+          <t>3 Stück</t>
         </is>
       </c>
       <c r="H10" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>4.79</v>
@@ -863,7 +863,7 @@
       <c r="K10" s="8" t="n"/>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Vorher Montageplatte messen: Passen 2 × 210 mm? Sonst eine dritte Schiene mitnehmen.</t>
+          <t>Eine Schiene je Ebene (3 Ebenen, Dok. 03). Neues Gehäuse 500 × 400 × 200: Montageplatte ca. 350 mm breit (Schätzung) – falls 210 mm zu kurz, eine 1-m-Schiene nehmen und kürzen.</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Bauhaus-Liste: Bestand aus der Projektmappe übernommen
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BNvKHpLgoxQiSKskTUqmN
</commit_message>
<xml_diff>
--- a/listen/Bauhaus_Einkaufsliste_MF70.xlsx
+++ b/listen/Bauhaus_Einkaufsliste_MF70.xlsx
@@ -613,7 +613,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>
@@ -665,7 +669,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>
@@ -717,7 +725,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>
@@ -769,7 +781,11 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>
@@ -1129,7 +1145,11 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>
@@ -1177,7 +1197,11 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>
@@ -1277,7 +1301,11 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr"/>
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
           <t>1 Elektro / Elektroinstallation</t>

</xml_diff>

<commit_message>
Bauhaus-Liste: Spiralschlauch 16 mm (Gesamtprüfung)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BNvKHpLgoxQiSKskTUqmN
</commit_message>
<xml_diff>
--- a/listen/Bauhaus_Einkaufsliste_MF70.xlsx
+++ b/listen/Bauhaus_Einkaufsliste_MF70.xlsx
@@ -1262,27 +1262,27 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Voltomat Spiralschlauch, max. Leitungs-Ø 8 mm, 2 m</t>
+          <t>Voltomat Kabelorganisierer (Spiralschlauch) 16 mm, schwarz</t>
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>12188841</v>
+        <v>12188827</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 2 m</t>
+          <t>1 Stk (Länge laut Shop widersprüchlich: 1,5 m oder 15 m)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>1 Stk</t>
+          <t>ca. 2 m</t>
         </is>
       </c>
       <c r="H18" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>4.25</v>
+        <v>7.62</v>
       </c>
       <c r="J18" s="7">
         <f>H18*I18</f>
@@ -1291,7 +1291,7 @@
       <c r="K18" s="8" t="n"/>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>Wenn das Bündel dicker als 8 mm wird, die nächstgrößere Variante nehmen.</t>
+          <t>Bündel ca. 13–15 mm (Schätzung), der 8-mm-Schlauch war zu eng. Länge auf der Packung prüfen: bei 15 m reicht 1 Packung. Zur Not 28-mm-Variante 12188834.</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Bauhaus-Liste: Gewiss-Kabelkanal gestrichen (Hager online)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BNvKHpLgoxQiSKskTUqmN
</commit_message>
<xml_diff>
--- a/listen/Bauhaus_Einkaufsliste_MF70.xlsx
+++ b/listen/Bauhaus_Einkaufsliste_MF70.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tipps für den Einkauf" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bauhaus-Einkaufsliste'!$A$5:$M$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bauhaus-Einkaufsliste'!$A$5:$M$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Bauhaus-Einkaufsliste'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1569,43 +1569,39 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Verdrahtungskanal im Schrank</t>
+          <t>Lötzinn</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Gewiss Verdrahtungskanal geschlitzt, 37,5 × 37,5 mm, 2 m, mit Deckel</t>
+          <t>Weller Elektroniklot bleifrei, 1 mm, 100 g</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>20748724</v>
+        <v>30448874</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 2 m</t>
+          <t>100 g</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>ca. 1 m</t>
+          <t>1 Rolle</t>
         </is>
       </c>
       <c r="H24" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>14.75</v>
+        <v>12.95</v>
       </c>
       <c r="J24" s="7">
         <f>H24*I24</f>
         <v/>
       </c>
       <c r="K24" s="8" t="n"/>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>Lässt sich mit Säge kürzen.</t>
-        </is>
-      </c>
+      <c r="L24" s="5" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -1621,39 +1617,43 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Lötzinn</t>
+          <t>USB-Kabel PC ↔ Arduino</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Weller Elektroniklot bleifrei, 1 mm, 100 g</t>
+          <t>Hama Verbindungskabel USB-A auf USB-B, 1,5 m</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>30448874</v>
+        <v>30568745</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>100 g</t>
+          <t>1 Stk</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>1 Rolle</t>
+          <t>2 Stk</t>
         </is>
       </c>
       <c r="H25" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>12.95</v>
+        <v>4.99</v>
       </c>
       <c r="J25" s="7">
         <f>H25*I25</f>
         <v/>
       </c>
       <c r="K25" s="8" t="n"/>
-      <c r="L25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Gibt es in der Multimedia-Abteilung. Eins als Reserve.</t>
+        </is>
+      </c>
       <c r="M25" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -1664,37 +1664,37 @@
       <c r="A26" s="4" t="inlineStr"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>1 Elektro / Elektroinstallation</t>
+          <t>2 Schrauben &amp; Eisenwaren</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>USB-Kabel PC ↔ Arduino</t>
+          <t>Zylinderschrauben M3 × 10</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Hama Verbindungskabel USB-A auf USB-B, 1,5 m</t>
+          <t>Suki Zylinderschraube DIN 912 M3 × 10, Innensechskant, verzinkt 8.8</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>30568745</v>
+        <v>10795755</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>1 Stk</t>
+          <t>16 Stk</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>2 Stk</t>
+          <t>ca. 12 Stk</t>
         </is>
       </c>
       <c r="H26" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>4.99</v>
+        <v>3.65</v>
       </c>
       <c r="J26" s="7">
         <f>H26*I26</f>
@@ -1703,7 +1703,7 @@
       <c r="K26" s="8" t="n"/>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>Gibt es in der Multimedia-Abteilung. Eins als Reserve.</t>
+          <t>Edelstahl (A2) gibt es bei Bauhaus in DIN 912 für M3–M5 nicht. Verzinkt 8.8 ist im trockenen Innenraum völlig in Ordnung und sogar fester.</t>
         </is>
       </c>
       <c r="M26" s="9" t="inlineStr">
@@ -1721,43 +1721,39 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Zylinderschrauben M3 × 10</t>
+          <t>Zylinderschrauben M3 × 16</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Suki Zylinderschraube DIN 912 M3 × 10, Innensechskant, verzinkt 8.8</t>
+          <t>Zylinderschraube DIN 912 M3 × 16, Innensechskant, verzinkt 8.8</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>10795755</v>
+        <v>21307483</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>16 Stk</t>
+          <t>10 Stk</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>ca. 12 Stk</t>
+          <t>ca. 8 Stk</t>
         </is>
       </c>
       <c r="H27" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>3.65</v>
+        <v>2.19</v>
       </c>
       <c r="J27" s="7">
         <f>H27*I27</f>
         <v/>
       </c>
       <c r="K27" s="8" t="n"/>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>Edelstahl (A2) gibt es bei Bauhaus in DIN 912 für M3–M5 nicht. Verzinkt 8.8 ist im trockenen Innenraum völlig in Ordnung und sogar fester.</t>
-        </is>
-      </c>
+      <c r="L27" s="5" t="inlineStr"/>
       <c r="M27" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -1773,39 +1769,43 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Zylinderschrauben M3 × 16</t>
+          <t>Zylinderschrauben M4 × 16</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Zylinderschraube DIN 912 M3 × 16, Innensechskant, verzinkt 8.8</t>
+          <t>Suki Zylinderschraube DIN 912 M4 × 16, Innensechskant, verzinkt 8.8</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>21307483</v>
+        <v>10795779</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>10 Stk</t>
+          <t>12 Stk</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>ca. 8 Stk</t>
+          <t>ca. 12 Stk</t>
         </is>
       </c>
       <c r="H28" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>2.19</v>
+        <v>3.1</v>
       </c>
       <c r="J28" s="7">
         <f>H28*I28</f>
         <v/>
       </c>
       <c r="K28" s="8" t="n"/>
-      <c r="L28" s="5" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Am Regal hängen meist auch M4 × 10 und M4 × 20 – bei Bedarf mitnehmen.</t>
+        </is>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -1821,16 +1821,16 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Zylinderschrauben M4 × 16</t>
+          <t>Zylinderschrauben M5 × 20</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Suki Zylinderschraube DIN 912 M4 × 16, Innensechskant, verzinkt 8.8</t>
+          <t>Zylinderschraube DIN 912 M5 × 20, Innensechskant, verzinkt 8.8</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>10795779</v>
+        <v>10795810</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
@@ -1839,14 +1839,14 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>ca. 12 Stk</t>
+          <t>ca. 8 Stk</t>
         </is>
       </c>
       <c r="H29" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>3.1</v>
+        <v>4.6</v>
       </c>
       <c r="J29" s="7">
         <f>H29*I29</f>
@@ -1855,7 +1855,7 @@
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>Am Regal hängen meist auch M4 × 10 und M4 × 20 – bei Bedarf mitnehmen.</t>
+          <t>M5 × 10 direkt daneben im Regal suchen, falls du kürzere brauchst.</t>
         </is>
       </c>
       <c r="M29" s="9" t="inlineStr">
@@ -1873,16 +1873,16 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Zylinderschrauben M5 × 20</t>
+          <t>Senkschrauben M4 (Aufspannplatte, Anschläge)</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Zylinderschraube DIN 912 M5 × 20, Innensechskant, verzinkt 8.8</t>
+          <t>Stabilit Senkkopfschraube DIN 7991 M4 × 16, Innensechskant, verzinkt 8.8</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>10795810</v>
+        <v>10801656</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
@@ -1891,14 +1891,14 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>ca. 8 Stk</t>
+          <t>ca. 10 Stk</t>
         </is>
       </c>
       <c r="H30" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
       <c r="J30" s="7">
         <f>H30*I30</f>
@@ -1907,7 +1907,7 @@
       <c r="K30" s="8" t="n"/>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>M5 × 10 direkt daneben im Regal suchen, falls du kürzere brauchst.</t>
+          <t>Größere Menge: Profi Depot DIN 7991 M4 × 20, 100 Stk, Art.-Nr. 20081793, 8,05 €.</t>
         </is>
       </c>
       <c r="M30" s="9" t="inlineStr">
@@ -1925,32 +1925,32 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Senkschrauben M4 (Aufspannplatte, Anschläge)</t>
+          <t>Muttern M3/M4/M5</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Stabilit Senkkopfschraube DIN 7991 M4 × 16, Innensechskant, verzinkt 8.8</t>
+          <t>BAUHAUS Mutternsortiment, verzinkt (u. a. 30 × M3, 25 × M4, 50 × M5)</t>
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>10801656</v>
+        <v>21996429</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>12 Stk</t>
+          <t>195 Stk in Box</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>ca. 10 Stk</t>
+          <t>1 Box</t>
         </is>
       </c>
       <c r="H31" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>4.9</v>
+        <v>12.25</v>
       </c>
       <c r="J31" s="7">
         <f>H31*I31</f>
@@ -1959,7 +1959,7 @@
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>Größere Menge: Profi Depot DIN 7991 M4 × 20, 100 Stk, Art.-Nr. 20081793, 8,05 €.</t>
+          <t>Wenn du schon Muttern hast: lieber Kleinpackungen M3/M4 am Schraubenregal.</t>
         </is>
       </c>
       <c r="M31" s="9" t="inlineStr">
@@ -1977,20 +1977,20 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Muttern M3/M4/M5</t>
+          <t>Unterlegscheiben M3/M4/M5</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>BAUHAUS Mutternsortiment, verzinkt (u. a. 30 × M3, 25 × M4, 50 × M5)</t>
+          <t>BAUHAUS Beilagscheiben-Sortiment, verzinkt (150 × M3, 150 × M4, 200 × M5 …)</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>21996429</v>
+        <v>21996960</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>195 Stk in Box</t>
+          <t>900 Stk in Box</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -2002,7 +2002,7 @@
         <v>1</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>12.25</v>
+        <v>17.9</v>
       </c>
       <c r="J32" s="7">
         <f>H32*I32</f>
@@ -2011,7 +2011,7 @@
       <c r="K32" s="8" t="n"/>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>Wenn du schon Muttern hast: lieber Kleinpackungen M3/M4 am Schraubenregal.</t>
+          <t>Wie oben – Kleinpackungen sind günstiger, wenn du nur wenige brauchst.</t>
         </is>
       </c>
       <c r="M32" s="9" t="inlineStr">
@@ -2029,32 +2029,32 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Unterlegscheiben M3/M4/M5</t>
+          <t>Fächerscheiben M4 (PE-Anschluss)</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>BAUHAUS Beilagscheiben-Sortiment, verzinkt (150 × M3, 150 × M4, 200 × M5 …)</t>
+          <t>Marinetech Fächerscheibe DIN 6798 A, Ø 4,3 mm, Edelstahl A4</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>21996960</v>
+        <v>23670996</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>900 Stk in Box</t>
+          <t>Einzelstück</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>1 Box</t>
+          <t>10 Stk</t>
         </is>
       </c>
       <c r="H33" s="5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>17.9</v>
+        <v>0.1</v>
       </c>
       <c r="J33" s="7">
         <f>H33*I33</f>
@@ -2063,7 +2063,7 @@
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>Wie oben – Kleinpackungen sind günstiger, wenn du nur wenige brauchst.</t>
+          <t>Wird einzeln verkauft – Stückzahl an der Kasse.</t>
         </is>
       </c>
       <c r="M33" s="9" t="inlineStr">
@@ -2081,16 +2081,16 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Fächerscheiben M4 (PE-Anschluss)</t>
+          <t>Fächerscheiben M5 (PE-Anschluss)</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Marinetech Fächerscheibe DIN 6798 A, Ø 4,3 mm, Edelstahl A4</t>
+          <t>Marinetech Fächerscheibe DIN 6798 A, Ø 5,3 mm, Edelstahl A4</t>
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>23670996</v>
+        <v>23671005</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -2106,7 +2106,7 @@
         <v>10</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="J34" s="7">
         <f>H34*I34</f>
@@ -2115,7 +2115,7 @@
       <c r="K34" s="8" t="n"/>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>Wird einzeln verkauft – Stückzahl an der Kasse.</t>
+          <t>Wie oben.</t>
         </is>
       </c>
       <c r="M34" s="9" t="inlineStr">
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Fächerscheiben M5 (PE-Anschluss)</t>
+          <t>Ersatz für Abstandsbolzen M3</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Marinetech Fächerscheibe DIN 6798 A, Ø 5,3 mm, Edelstahl A4</t>
+          <t>Profi Depot Gewindestange M3, 1 m, verzinkt</t>
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>23671005</v>
+        <v>10827348</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Einzelstück</t>
+          <t>1 Stk, 1 m</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>10 Stk</t>
+          <t>1 Stk</t>
         </is>
       </c>
       <c r="H35" s="5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.12</v>
+        <v>0.85</v>
       </c>
       <c r="J35" s="7">
         <f>H35*I35</f>
@@ -2167,7 +2167,7 @@
       <c r="K35" s="8" t="n"/>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>Wie oben.</t>
+          <t>Abstandsbolzen hat Bauhaus nicht. Stange auf Länge sägen und mit Muttern kontern.</t>
         </is>
       </c>
       <c r="M35" s="9" t="inlineStr">
@@ -2185,32 +2185,32 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Ersatz für Abstandsbolzen M3</t>
+          <t>Gerätefüße für den Schaltschrank</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Profi Depot Gewindestange M3, 1 m, verzinkt</t>
+          <t>Stabilit Anti-Vibration-Pad, Gummi, schwarz, 70 × 35 mm</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>10827348</v>
+        <v>22487485</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 1 m</t>
+          <t>2 Stk</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>1 Stk</t>
+          <t>4 Stk</t>
         </is>
       </c>
       <c r="H36" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I36" s="7" t="n">
-        <v>0.85</v>
+        <v>6.25</v>
       </c>
       <c r="J36" s="7">
         <f>H36*I36</f>
@@ -2219,7 +2219,7 @@
       <c r="K36" s="8" t="n"/>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>Abstandsbolzen hat Bauhaus nicht. Stange auf Länge sägen und mit Muttern kontern.</t>
+          <t>Ist eher groß – alternativ im Markt nach selbstklebenden Gummipuffern (Möbel-/Filzgleiter-Regal) schauen.</t>
         </is>
       </c>
       <c r="M36" s="9" t="inlineStr">
@@ -2232,37 +2232,37 @@
       <c r="A37" s="4" t="inlineStr"/>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2 Schrauben &amp; Eisenwaren</t>
+          <t>3 Metall- &amp; Kunststoffprofile</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Gerätefüße für den Schaltschrank</t>
+          <t>Anschlagkanten Aufspannplatte</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Stabilit Anti-Vibration-Pad, Gummi, schwarz, 70 × 35 mm</t>
+          <t>Kantoflex Winkelprofil Alu 15,5 × 15,5 × 1,5 mm, 1 m</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>22487485</v>
+        <v>10522241</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>2 Stk</t>
+          <t>1 Stk, 1 m</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>4 Stk</t>
+          <t>1 Stk</t>
         </is>
       </c>
       <c r="H37" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>6.25</v>
+        <v>2.95</v>
       </c>
       <c r="J37" s="7">
         <f>H37*I37</f>
@@ -2271,7 +2271,7 @@
       <c r="K37" s="8" t="n"/>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>Ist eher groß – alternativ im Markt nach selbstklebenden Gummipuffern (Möbel-/Filzgleiter-Regal) schauen.</t>
+          <t>1,5 statt 2 mm Wandstärke – reicht für Anschläge.</t>
         </is>
       </c>
       <c r="M37" s="9" t="inlineStr">
@@ -2289,32 +2289,32 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Anschlagkanten Aufspannplatte</t>
+          <t>Endschalterhalter, Schaltnocken, Kamerahalter</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Kantoflex Winkelprofil Alu 15,5 × 15,5 × 1,5 mm, 1 m</t>
+          <t>Kantoflex Winkelprofil Alu 20 × 20 × 1,5 mm, eloxiert, 2 m</t>
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>10522241</v>
+        <v>10507637</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 1 m</t>
+          <t>1 Stk, 2 m</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>1 Stk</t>
+          <t>ca. 1 m</t>
         </is>
       </c>
       <c r="H38" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>2.95</v>
+        <v>6.65</v>
       </c>
       <c r="J38" s="7">
         <f>H38*I38</f>
@@ -2323,7 +2323,7 @@
       <c r="K38" s="8" t="n"/>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>1,5 statt 2 mm Wandstärke – reicht für Anschläge.</t>
+          <t>Gibt es nur als 2-m-Stange; im Markt nach 1-m-Variante fragen.</t>
         </is>
       </c>
       <c r="M38" s="9" t="inlineStr">
@@ -2341,43 +2341,39 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Endschalterhalter, Schaltnocken, Kamerahalter</t>
+          <t>Kamerahalter</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Kantoflex Winkelprofil Alu 20 × 20 × 1,5 mm, eloxiert, 2 m</t>
+          <t>Kantoflex Flachprofil Alu 20 × 5 mm, eloxiert, 1 m</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>10507637</v>
+        <v>10520009</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 2 m</t>
+          <t>1 Stk, 1 m</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>ca. 1 m</t>
+          <t>1 Stk</t>
         </is>
       </c>
       <c r="H39" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>6.65</v>
+        <v>5.8</v>
       </c>
       <c r="J39" s="7">
         <f>H39*I39</f>
         <v/>
       </c>
       <c r="K39" s="8" t="n"/>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>Gibt es nur als 2-m-Stange; im Markt nach 1-m-Variante fragen.</t>
-        </is>
-      </c>
+      <c r="L39" s="5" t="inlineStr"/>
       <c r="M39" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -2393,16 +2389,16 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Kamerahalter</t>
+          <t>Selbstbau-Nutensteine</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Kantoflex Flachprofil Alu 20 × 5 mm, eloxiert, 1 m</t>
+          <t>Kantoflex Flachprofil Stahl blank 10 × 4 mm, 1 m</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>10520009</v>
+        <v>10526797</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
@@ -2418,14 +2414,18 @@
         <v>1</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>5.8</v>
+        <v>2.65</v>
       </c>
       <c r="J40" s="7">
         <f>H40*I40</f>
         <v/>
       </c>
       <c r="K40" s="8" t="n"/>
-      <c r="L40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Vorher die T-Nut der MF 70 nachmessen (12 × 6 × 5 mm).</t>
+        </is>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -2436,37 +2436,37 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>3 Metall- &amp; Kunststoffprofile</t>
+          <t>4 Holz &amp; Zuschnitt</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Selbstbau-Nutensteine</t>
+          <t>Opferplatte / Unterbau Aufspannplatte</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Kantoflex Flachprofil Stahl blank 10 × 4 mm, 1 m</t>
+          <t>MDF-Platte nach Maß, natur, 12 mm (Preis je m²)</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>10526797</v>
+        <v>14471013</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 1 m</t>
+          <t>Zuschnitt nach Maß</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>1 Stk</t>
+          <t>2 × 250 × 120 mm = 0,06 m²</t>
         </is>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1</v>
+        <v>0.06</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>2.65</v>
+        <v>15.85</v>
       </c>
       <c r="J41" s="7">
         <f>H41*I41</f>
@@ -2475,7 +2475,7 @@
       <c r="K41" s="8" t="n"/>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>Vorher die T-Nut der MF 70 nachmessen (12 × 6 × 5 mm).</t>
+          <t>Preis ist pro m². Am Zuschnitt fragen, ob es eine Mindestmenge oder Schnittkosten gibt – oft lohnt sich ein Reststück. Maße erst nach der Freiraummessung festlegen.</t>
         </is>
       </c>
       <c r="M41" s="9" t="inlineStr">
@@ -2493,32 +2493,32 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Opferplatte / Unterbau Aufspannplatte</t>
+          <t>Probestücke zum Fräsen</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>MDF-Platte nach Maß, natur, 12 mm (Preis je m²)</t>
+          <t>Rechteckleiste Buche, 40 × 20 mm, 1 m</t>
         </is>
       </c>
       <c r="E42" s="6" t="n">
-        <v>14471013</v>
+        <v>14610733</v>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Zuschnitt nach Maß</t>
+          <t>1 Stk, 1 m</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>2 × 250 × 120 mm = 0,06 m²</t>
+          <t>2 Stk</t>
         </is>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.06</v>
+        <v>2</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>15.85</v>
+        <v>8.35</v>
       </c>
       <c r="J42" s="7">
         <f>H42*I42</f>
@@ -2527,7 +2527,7 @@
       <c r="K42" s="8" t="n"/>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>Preis ist pro m². Am Zuschnitt fragen, ob es eine Mindestmenge oder Schnittkosten gibt – oft lohnt sich ein Reststück. Maße erst nach der Freiraummessung festlegen.</t>
+          <t>In 100-mm-Stücke sägen.</t>
         </is>
       </c>
       <c r="M42" s="9" t="inlineStr">
@@ -2540,37 +2540,37 @@
       <c r="A43" s="4" t="inlineStr"/>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>4 Holz &amp; Zuschnitt</t>
+          <t>3 Metall- &amp; Kunststoffprofile</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Probestücke zum Fräsen</t>
+          <t>Späneschutz (Polycarbonat)</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Rechteckleiste Buche, 40 × 20 mm, 1 m</t>
+          <t>Kunstglas Polycarbonat farblos, 4 mm, 500 × 1000 mm</t>
         </is>
       </c>
       <c r="E43" s="6" t="n">
-        <v>14610733</v>
+        <v>29619304</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>1 Stk, 1 m</t>
+          <t>1 Platte</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>2 Stk</t>
+          <t>ca. 200 × 150 mm</t>
         </is>
       </c>
       <c r="H43" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>8.35</v>
+        <v>28.75</v>
       </c>
       <c r="J43" s="7">
         <f>H43*I43</f>
@@ -2579,7 +2579,7 @@
       <c r="K43" s="8" t="n"/>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>In 100-mm-Stücke sägen.</t>
+          <t>3 mm gibt es nicht – 4 mm geht auch und ist stabiler. Kein Acrylglas (PMMA) nehmen, das splittert. Die Platte ist viel zu groß: im Markt nach Zuschnitt oder Reststück fragen.</t>
         </is>
       </c>
       <c r="M43" s="9" t="inlineStr">
@@ -2592,48 +2592,44 @@
       <c r="A44" s="4" t="inlineStr"/>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>3 Metall- &amp; Kunststoffprofile</t>
+          <t>5 Farben, Kleben, Pflege</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Späneschutz (Polycarbonat)</t>
+          <t>Werkstück spannen (flache Hölzer)</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Kunstglas Polycarbonat farblos, 4 mm, 500 × 1000 mm</t>
+          <t>Duck Smart doppelseitiges Teppichband, 50 mm × 5 m</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>29619304</v>
+        <v>26335957</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>1 Platte</t>
+          <t>1 Rolle</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>ca. 200 × 150 mm</t>
+          <t>1 Rolle</t>
         </is>
       </c>
       <c r="H44" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>28.75</v>
+        <v>2.95</v>
       </c>
       <c r="J44" s="7">
         <f>H44*I44</f>
         <v/>
       </c>
       <c r="K44" s="8" t="n"/>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>3 mm gibt es nicht – 4 mm geht auch und ist stabiler. Kein Acrylglas (PMMA) nehmen, das splittert. Die Platte ist viel zu groß: im Markt nach Zuschnitt oder Reststück fragen.</t>
-        </is>
-      </c>
+      <c r="L44" s="5" t="inlineStr"/>
       <c r="M44" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -2649,39 +2645,43 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Werkstück spannen (flache Hölzer)</t>
+          <t>Kontrastfarbe Opferplatte / Passmarken für die Kamera</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Duck Smart doppelseitiges Teppichband, 50 mm × 5 m</t>
+          <t>Dupli-Color Aerosol Art Sprühlack RAL 9005 tiefschwarz matt, 400 ml</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>26335957</v>
+        <v>15073128</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>1 Rolle</t>
+          <t>400 ml</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>1 Rolle</t>
+          <t>1 Dose</t>
         </is>
       </c>
       <c r="H45" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>2.95</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="J45" s="7">
         <f>H45*I45</f>
         <v/>
       </c>
       <c r="K45" s="8" t="n"/>
-      <c r="L45" s="5" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>Matt ist wichtig, damit die Kamera keine Spiegelungen sieht.</t>
+        </is>
+      </c>
       <c r="M45" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -2697,43 +2697,39 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Kontrastfarbe Opferplatte / Passmarken für die Kamera</t>
+          <t>Schmierung der Führungen</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Dupli-Color Aerosol Art Sprühlack RAL 9005 tiefschwarz matt, 400 ml</t>
+          <t>Profi Depot Feinmechaniköl, 150 ml</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>15073128</v>
+        <v>22829078</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>400 ml</t>
+          <t>150 ml</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>1 Dose</t>
+          <t>1 Flasche</t>
         </is>
       </c>
       <c r="H46" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>9.949999999999999</v>
+        <v>4.79</v>
       </c>
       <c r="J46" s="7">
         <f>H46*I46</f>
         <v/>
       </c>
       <c r="K46" s="8" t="n"/>
-      <c r="L46" s="5" t="inlineStr">
-        <is>
-          <t>Matt ist wichtig, damit die Kamera keine Spiegelungen sieht.</t>
-        </is>
-      </c>
+      <c r="L46" s="5" t="inlineStr"/>
       <c r="M46" s="9" t="inlineStr">
         <is>
           <t>bauhaus.info</t>
@@ -2749,32 +2745,32 @@
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Schmierung der Führungen</t>
+          <t>Späne wegpinseln</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Profi Depot Feinmechaniköl, 150 ml</t>
+          <t>Flachpinsel 30 mm, Mischborsten</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>22829078</v>
+        <v>25873454</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>150 ml</t>
+          <t>1 Stk</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>1 Flasche</t>
+          <t>1 Stk</t>
         </is>
       </c>
       <c r="H47" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>4.79</v>
+        <v>2.35</v>
       </c>
       <c r="J47" s="7">
         <f>H47*I47</f>
@@ -2789,72 +2785,24 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr"/>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>5 Farben, Kleben, Pflege</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Späne wegpinseln</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Flachpinsel 30 mm, Mischborsten</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="n">
-        <v>25873454</v>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>1 Stk</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>1 Stk</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I48" s="7" t="n">
-        <v>2.35</v>
-      </c>
-      <c r="J48" s="7">
-        <f>H48*I48</f>
-        <v/>
-      </c>
-      <c r="K48" s="8" t="n"/>
-      <c r="L48" s="5" t="inlineStr"/>
-      <c r="M48" s="9" t="inlineStr">
-        <is>
-          <t>bauhaus.info</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="I49" s="10" t="inlineStr">
+      <c r="I48" s="10" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="J49" s="11">
-        <f>SUM(J6:J48)</f>
-        <v/>
-      </c>
-      <c r="K49" s="11">
-        <f>SUM(K6:K48)</f>
+      <c r="J48" s="11">
+        <f>SUM(J6:J47)</f>
+        <v/>
+      </c>
+      <c r="K48" s="11">
+        <f>SUM(K6:K47)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:M48"/>
+  <autoFilter ref="A5:M47"/>
   <dataValidations count="1">
-    <dataValidation sqref="A6:A48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A6:A47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2901,7 +2849,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId43"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Bauhaus-Liste: Hinweise USB innen und Flachsteckhülsen (Verdrahtungsliste Rev. G)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BNvKHpLgoxQiSKskTUqmN
</commit_message>
<xml_diff>
--- a/listen/Bauhaus_Einkaufsliste_MF70.xlsx
+++ b/listen/Bauhaus_Einkaufsliste_MF70.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preise: Online-Preise von bauhaus.info (Stand Dokument 04: 26.10.2026, Liste erzeugt am 26.10.2026). Im Markt können Preis und Bestand abweichen.</t>
+          <t>Preise: Online-Preise von bauhaus.info (Stand Dokument 04: 27.10.2026, Liste erzeugt am 27.10.2026). Im Markt können Preis und Bestand abweichen.</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       <c r="K14" s="8" t="n"/>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Im Set sind u. a. Ringkabelschuhe – auf der Packung prüfen, ob Loch für M4/M5 dabei ist. Wenn nicht: einzelne Ringkabelschuhe am Elektroregal suchen.</t>
+          <t>Im Set sind u. a. Ringkabelschuhe – auf der Packung prüfen, ob Loch für M4/M5 dabei ist. Rev. G: Prüfen, ob isolierte Flachsteckhülsen 6,3 mm für 1,5 mm² dabei sind (nur nötig, falls -X0 Flachstecker hat). Wenn nicht: einzelne Ringkabelschuhe am Elektroregal suchen.</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
@@ -1651,7 +1651,7 @@
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>Gibt es in der Multimedia-Abteilung. Eins als Reserve.</t>
+          <t>Gibt es in der Multimedia-Abteilung. Eins für außen (PC → Schrank), eins als Reserve. Innen im Schrank passt A auf B nicht (Durchführung hat innen B-Buchse) – dafür B-auf-B-Kabel online (Materialliste).</t>
         </is>
       </c>
       <c r="M25" s="9" t="inlineStr">

</xml_diff>